<commit_message>
TRM template: update DataValid brand list to TRM brands (12) — user-edited, dropdowns preserved
</commit_message>
<xml_diff>
--- a/public/air-request-template_TRM.xlsx
+++ b/public/air-request-template_TRM.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D250F3B-9ACD-4FAE-A37A-AA6A37187591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AE3193E-3866-473D-A7FC-3C76FA7A89FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="163">
   <si>
     <t>LOGISTICS</t>
   </si>
@@ -164,9 +164,6 @@
     <t>Melbourne</t>
   </si>
   <si>
-    <t>TOMMY BAHAMA</t>
-  </si>
-  <si>
     <t>G4</t>
   </si>
   <si>
@@ -197,9 +194,6 @@
     <t>Amsterdam</t>
   </si>
   <si>
-    <t>LSKD</t>
-  </si>
-  <si>
     <t>CLAIM</t>
   </si>
   <si>
@@ -212,9 +206,6 @@
     <t>O'hare(ORD)</t>
   </si>
   <si>
-    <t>PETER MILLAR LLC</t>
-  </si>
-  <si>
     <t>PROCUREMENT</t>
   </si>
   <si>
@@ -299,96 +290,24 @@
     <t>Tokyo</t>
   </si>
   <si>
-    <t>WORKWEAR OUTFITTERS LLC</t>
-  </si>
-  <si>
     <t>OMNI APPARATECH INC.</t>
   </si>
   <si>
-    <t>JR286 INTERNATIONATIONAL, LLC</t>
-  </si>
-  <si>
-    <t>FANATICS, INC.</t>
-  </si>
-  <si>
-    <t>TOMMY JOHN, INC.</t>
-  </si>
-  <si>
-    <t>BYLT LLC</t>
-  </si>
-  <si>
-    <t>YETI COOLERS</t>
-  </si>
-  <si>
-    <t>BCS (BRANDED CUSTOM SPORTSWEAR)</t>
-  </si>
-  <si>
-    <t>LULULEMON ATHLETICA CANADA INC.</t>
-  </si>
-  <si>
     <t>5.11 INC.</t>
   </si>
   <si>
-    <t>CENTER</t>
-  </si>
-  <si>
-    <t>RUDIS</t>
-  </si>
-  <si>
-    <t>OXFORD INDUSTRIES INC</t>
-  </si>
-  <si>
-    <t>BOMBAS LLC</t>
-  </si>
-  <si>
-    <t>GYALSUNG HEADQUARTERS</t>
-  </si>
-  <si>
-    <t>SRICHAN CHAIWILAI</t>
-  </si>
-  <si>
     <t>LOLE BRANDS CANADA ULC</t>
   </si>
   <si>
-    <t>THE S GROUP, INC.,</t>
-  </si>
-  <si>
-    <t>AMER SPORTS SOURCING LIMITED</t>
-  </si>
-  <si>
     <t>PRIME SOLUTION ASIA</t>
   </si>
   <si>
-    <t>DICK S SPORTING</t>
-  </si>
-  <si>
     <t>BRIO MAX LIMITED</t>
   </si>
   <si>
-    <t>ACUSHNET COMPANY</t>
-  </si>
-  <si>
-    <t>SITI KHADIJAH APPAREL SDN BHD</t>
-  </si>
-  <si>
     <t>O'NEILLS IRISH INTERNATIONAL SPORTS CO.,LTD</t>
   </si>
   <si>
-    <t>LAAINAM CHAIPORNKAEW</t>
-  </si>
-  <si>
-    <t>NIKE</t>
-  </si>
-  <si>
-    <t>FOX GOLF</t>
-  </si>
-  <si>
-    <t>ASICS CORPORATION</t>
-  </si>
-  <si>
-    <t>LEGENDS</t>
-  </si>
-  <si>
     <t>NYK</t>
   </si>
   <si>
@@ -551,9 +470,6 @@
     <t>VIETNAM</t>
   </si>
   <si>
-    <t>G/FORE</t>
-  </si>
-  <si>
     <t>DRIFIT SLEEVES</t>
   </si>
   <si>
@@ -582,6 +498,24 @@
   </si>
   <si>
     <t>TANK</t>
+  </si>
+  <si>
+    <t>INDYGENA.COM / APROPOZ.COM</t>
+  </si>
+  <si>
+    <t>MODATEX</t>
+  </si>
+  <si>
+    <t>PERRY ELLIS INTERNATIONAL</t>
+  </si>
+  <si>
+    <t>เรดวูดส์ อินเตอร์เนชั่นแนล บจ.</t>
+  </si>
+  <si>
+    <t>กรอสเวล บจก.</t>
+  </si>
+  <si>
+    <t>นันยางการ์เม้นท์  บจก.</t>
   </si>
 </sst>
 </file>
@@ -967,7 +901,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="MASTER_BRAND" displayName="MASTER_BRAND" ref="A1:A35" headerRowCount="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="MASTER_BRAND" displayName="MASTER_BRAND" ref="A1:A13" headerRowCount="0">
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="BRAND_NAME"/>
   </tableColumns>
@@ -1351,7 +1285,7 @@
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A1" s="34" t="s">
-        <v>121</v>
+        <v>94</v>
       </c>
       <c r="B1" s="34"/>
       <c r="C1" s="34"/>
@@ -2317,8 +2251,8 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
-        <v>99</v>
+      <c r="A2" t="s">
+        <v>88</v>
       </c>
       <c r="C2" t="s">
         <v>35</v>
@@ -2327,19 +2261,19 @@
         <v>36</v>
       </c>
       <c r="G2" s="27" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H2" s="27"/>
       <c r="J2" s="28" t="s">
         <v>38</v>
       </c>
       <c r="L2" s="28" t="s">
-        <v>122</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="27" t="s">
-        <v>112</v>
+      <c r="A3" t="s">
+        <v>91</v>
       </c>
       <c r="C3" t="s">
         <v>39</v>
@@ -2348,19 +2282,19 @@
         <v>40</v>
       </c>
       <c r="G3" s="27" t="s">
-        <v>175</v>
+        <v>147</v>
       </c>
       <c r="H3" s="27"/>
       <c r="J3" s="29" t="s">
         <v>41</v>
       </c>
       <c r="L3" s="28" t="s">
-        <v>123</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="27" t="s">
-        <v>108</v>
+      <c r="A4" t="s">
+        <v>157</v>
       </c>
       <c r="C4" t="s">
         <v>42</v>
@@ -2369,519 +2303,453 @@
         <v>43</v>
       </c>
       <c r="G4" s="27" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="H4" s="27"/>
       <c r="J4" s="28" t="s">
         <v>44</v>
       </c>
       <c r="L4" s="29" t="s">
-        <v>124</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="27" t="s">
-        <v>118</v>
+      <c r="A5" t="s">
+        <v>89</v>
       </c>
       <c r="C5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E5" t="s">
         <v>46</v>
       </c>
-      <c r="E5" t="s">
-        <v>47</v>
-      </c>
       <c r="G5" s="27" t="s">
-        <v>176</v>
+        <v>148</v>
       </c>
       <c r="H5" s="27"/>
       <c r="J5" s="29" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L5" s="29" t="s">
-        <v>125</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" s="27" t="s">
-        <v>97</v>
+      <c r="A6" t="s">
+        <v>158</v>
       </c>
       <c r="G6" s="27" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="H6" s="27"/>
       <c r="J6" s="28" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="L6" s="28" t="s">
-        <v>126</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="27" t="s">
-        <v>103</v>
+      <c r="A7" t="s">
+        <v>87</v>
       </c>
       <c r="G7" s="27" t="s">
-        <v>177</v>
+        <v>149</v>
       </c>
       <c r="H7" s="27"/>
       <c r="J7" s="29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="L7" s="29" t="s">
-        <v>127</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" s="27" t="s">
-        <v>111</v>
+      <c r="A8" t="s">
+        <v>92</v>
       </c>
       <c r="G8" s="27" t="s">
-        <v>178</v>
+        <v>150</v>
       </c>
       <c r="H8" s="27"/>
       <c r="J8" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="L8" s="28" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>159</v>
+      </c>
+      <c r="C9" t="s">
         <v>55</v>
       </c>
-      <c r="L8" s="28" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="27" t="s">
-        <v>95</v>
-      </c>
-      <c r="C9" t="s">
-        <v>57</v>
-      </c>
       <c r="G9" s="27" t="s">
-        <v>179</v>
+        <v>151</v>
       </c>
       <c r="H9" s="27"/>
       <c r="J9" s="29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="L9" s="28" t="s">
-        <v>129</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" s="27" t="s">
-        <v>100</v>
+      <c r="A10" t="s">
+        <v>90</v>
       </c>
       <c r="C10" t="s">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="G10" s="27" t="s">
-        <v>180</v>
+        <v>152</v>
       </c>
       <c r="H10" s="27"/>
       <c r="J10" s="28" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="L10" s="28" t="s">
-        <v>130</v>
+        <v>103</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11" s="27" t="s">
-        <v>110</v>
+      <c r="A11" t="s">
+        <v>160</v>
       </c>
       <c r="C11" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G11" s="27" t="s">
-        <v>181</v>
+        <v>153</v>
       </c>
       <c r="H11" s="27"/>
       <c r="J11" s="28" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="L11" s="29" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>93</v>
+        <v>161</v>
       </c>
       <c r="C12" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G12" s="27" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="H12" s="27"/>
       <c r="J12" s="28" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="L12" s="30" t="s">
-        <v>132</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>117</v>
+        <v>162</v>
       </c>
       <c r="C13" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="G13" s="27" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H13" s="27"/>
       <c r="J13" s="31" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="L13" t="s">
-        <v>133</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>104</v>
-      </c>
       <c r="G14" s="27" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H14" s="27"/>
       <c r="J14" s="28" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="L14" t="s">
-        <v>134</v>
+        <v>107</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>92</v>
-      </c>
       <c r="G15" s="27" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H15" s="27"/>
       <c r="J15" s="29" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="L15" t="s">
-        <v>135</v>
+        <v>108</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>115</v>
-      </c>
       <c r="G16" s="27" t="s">
         <v>37</v>
       </c>
       <c r="H16" s="27"/>
       <c r="J16" s="28" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="L16" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>119</v>
-      </c>
+        <v>109</v>
+      </c>
+    </row>
+    <row r="17" spans="7:12" x14ac:dyDescent="0.25">
       <c r="G17" s="27" t="s">
-        <v>182</v>
+        <v>154</v>
       </c>
       <c r="H17" s="27"/>
       <c r="J17" s="29" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="L17" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>106</v>
-      </c>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="18" spans="7:12" x14ac:dyDescent="0.25">
       <c r="G18" s="27" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="H18" s="27"/>
       <c r="J18" s="28" t="s">
+        <v>73</v>
+      </c>
+      <c r="L18" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="19" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="G19" t="s">
+        <v>155</v>
+      </c>
+      <c r="J19" s="29" t="s">
+        <v>74</v>
+      </c>
+      <c r="L19" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="20" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="G20" t="s">
+        <v>51</v>
+      </c>
+      <c r="J20" s="28" t="s">
+        <v>75</v>
+      </c>
+      <c r="L20" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="21" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="G21" t="s">
+        <v>156</v>
+      </c>
+      <c r="J21" s="29" t="s">
         <v>76</v>
       </c>
-      <c r="L18" t="s">
+      <c r="L21" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="22" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J22" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="L22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="23" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J23" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="L23" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="24" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J24" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="L24" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="25" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J25" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="L25" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="26" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J26" s="28" t="s">
+        <v>81</v>
+      </c>
+      <c r="L26" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="27" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J27" s="29" t="s">
+        <v>82</v>
+      </c>
+      <c r="L27" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="28" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J28" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="L28" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="29" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J29" s="29" t="s">
+        <v>84</v>
+      </c>
+      <c r="L29" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="30" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J30" s="29" t="s">
+        <v>85</v>
+      </c>
+      <c r="L30" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="31" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J31" s="32" t="s">
+        <v>86</v>
+      </c>
+      <c r="L31" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="32" spans="7:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L32" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="33" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L33" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="34" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L34" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="35" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L35" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="36" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L36" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="37" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L37" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="38" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L38" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="39" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L39" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="40" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L40" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="41" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L41" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="42" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L42" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="43" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L43" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="44" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L44" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="45" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L45" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>56</v>
-      </c>
-      <c r="G19" t="s">
-        <v>183</v>
-      </c>
-      <c r="J19" s="29" t="s">
-        <v>77</v>
-      </c>
-      <c r="L19" t="s">
+    <row r="46" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L46" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>98</v>
-      </c>
-      <c r="G20" t="s">
-        <v>52</v>
-      </c>
-      <c r="J20" s="28" t="s">
-        <v>78</v>
-      </c>
-      <c r="L20" t="s">
+    <row r="47" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L47" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>116</v>
-      </c>
-      <c r="G21" t="s">
-        <v>184</v>
-      </c>
-      <c r="J21" s="29" t="s">
-        <v>79</v>
-      </c>
-      <c r="L21" t="s">
+    <row r="48" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L48" t="s">
         <v>141</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>91</v>
-      </c>
-      <c r="J22" s="28" t="s">
-        <v>80</v>
-      </c>
-      <c r="L22" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>114</v>
-      </c>
-      <c r="J23" s="28" t="s">
-        <v>81</v>
-      </c>
-      <c r="L23" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>102</v>
-      </c>
-      <c r="J24" s="28" t="s">
-        <v>82</v>
-      </c>
-      <c r="L24" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>61</v>
-      </c>
-      <c r="J25" s="29" t="s">
-        <v>83</v>
-      </c>
-      <c r="L25" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>109</v>
-      </c>
-      <c r="J26" s="28" t="s">
-        <v>84</v>
-      </c>
-      <c r="L26" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>101</v>
-      </c>
-      <c r="J27" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="L27" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>113</v>
-      </c>
-      <c r="J28" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="L28" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>105</v>
-      </c>
-      <c r="J29" s="29" t="s">
-        <v>87</v>
-      </c>
-      <c r="L29" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>107</v>
-      </c>
-      <c r="J30" s="29" t="s">
-        <v>88</v>
-      </c>
-      <c r="L30" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>45</v>
-      </c>
-      <c r="J31" s="32" t="s">
-        <v>89</v>
-      </c>
-      <c r="L31" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>94</v>
-      </c>
-      <c r="L32" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>90</v>
-      </c>
-      <c r="L33" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>96</v>
-      </c>
-      <c r="L34" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>174</v>
-      </c>
-      <c r="L35" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="L36" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="L37" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="L38" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="L39" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="L40" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="L41" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="L42" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="L43" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="L44" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="L45" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="46" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="L46" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="L47" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="48" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="L48" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="49" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L49" t="s">
-        <v>169</v>
+        <v>142</v>
       </c>
     </row>
     <row r="50" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L50" t="s">
-        <v>170</v>
+        <v>143</v>
       </c>
     </row>
     <row r="51" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L51" t="s">
-        <v>171</v>
+        <v>144</v>
       </c>
     </row>
     <row r="52" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L52" t="s">
-        <v>172</v>
+        <v>145</v>
       </c>
     </row>
     <row r="53" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L53" t="s">
-        <v>173</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>